<commit_message>
V6 : SBF 120 - 85 actions - Excel avec graphiques
</commit_message>
<xml_diff>
--- a/HALAL_QUANT_CAC40_V5.xlsx
+++ b/HALAL_QUANT_CAC40_V5.xlsx
@@ -347,12 +347,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Graphiques'!$A$8:$A$23</f>
+              <f>'Graphiques'!$A$8:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Graphiques'!$B$8:$B$23</f>
+              <f>'Graphiques'!$B$8:$B$24</f>
             </numRef>
           </val>
         </ser>
@@ -939,10 +939,10 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>109.5</v>
+        <v>107.8</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>316</v>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>29.78</v>
+        <v>29.66</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>2.9</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1908</v>
+        <v>1873</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>44.4</v>
+        <v>43.4</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>25.2</v>
@@ -1185,7 +1185,7 @@
         <v>1.2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>0</v>
@@ -1233,13 +1233,13 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>361.25</v>
+        <v>353.65</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>31.6</v>
+        <v>31</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>18</v>
@@ -1254,10 +1254,10 @@
         <v>0.88</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>0</v>
@@ -1283,12 +1283,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>SU.PA</t>
+          <t>AI.PA</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Schneider Electric</t>
+          <t>Air Liquide</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1305,31 +1305,31 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>252.2</v>
+        <v>170.88</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>31.7</v>
+        <v>28</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>164</v>
+        <v>217</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>15.6</v>
+        <v>13.4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>10.4</v>
+        <v>13.1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4.2</v>
+        <v>-3.4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1.03</v>
+        <v>0.72</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>14</v>
+        <v>13.8</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>3.3</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>0</v>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr">
         <is>
-          <t>Specialty Industrial Machinery</t>
+          <t>Specialty Chemicals</t>
         </is>
       </c>
       <c r="T8" s="4" t="inlineStr"/>
@@ -1355,12 +1355,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>AI.PA</t>
+          <t>SU.PA</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Air Liquide</t>
+          <t>Schneider Electric</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
@@ -1377,31 +1377,31 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>169.16</v>
+        <v>248</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>27.7</v>
+        <v>31.1</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>221</v>
+        <v>165</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>13.4</v>
+        <v>15.6</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>13.1</v>
+        <v>10.4</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>-3.4</v>
+        <v>4.2</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.72</v>
+        <v>1.03</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>14</v>
+        <v>14.3</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>4.1</v>
+        <v>3.3</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>0</v>
@@ -1414,12 +1414,12 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>Specialty Chemicals</t>
+          <t>Specialty Industrial Machinery</t>
         </is>
       </c>
       <c r="T9" s="4" t="inlineStr"/>
@@ -1449,10 +1449,10 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>209.5</v>
+        <v>204.7</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>42.1</v>
+        <v>41.2</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>190</v>
@@ -1470,7 +1470,7 @@
         <v>0.55</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>14.8</v>
+        <v>15.2</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>3.7</v>
@@ -1521,13 +1521,13 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>306.1</v>
+        <v>304.4</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>55.6</v>
@@ -1597,10 +1597,10 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>137.6</v>
+        <v>136.85</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>29.3</v>
+        <v>29.1</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>172</v>
@@ -1618,10 +1618,10 @@
         <v>0.91</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>0</v>
@@ -1669,13 +1669,13 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>18.61</v>
+        <v>18.5</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I13" s="4" t="n">
         <v>13.3</v>
@@ -1690,10 +1690,10 @@
         <v>0.47</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>16.8</v>
+        <v>16.9</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>0</v>
@@ -1741,13 +1741,13 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>28.91</v>
+        <v>28.61</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>192.7</v>
+        <v>178.8</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I14" s="4" t="n">
         <v>1</v>
@@ -1762,10 +1762,10 @@
         <v>1.37</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>0</v>
@@ -1813,13 +1813,13 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>76.41</v>
+        <v>76.39</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>19</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="I15" s="4" t="n">
         <v>6.7</v>
@@ -1885,13 +1885,13 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>255.1</v>
+        <v>253.8</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>31.4</v>
+        <v>31.2</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>21.1</v>
@@ -1906,7 +1906,7 @@
         <v>0.13</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="N16" s="5" t="n">
         <v>8.6</v>
@@ -1961,13 +1961,13 @@
         </is>
       </c>
       <c r="F17" s="5" t="n">
-        <v>171.3</v>
+        <v>168.38</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>21.6</v>
@@ -1982,10 +1982,10 @@
         <v>0.83</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>10.5</v>
+        <v>10.7</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="O17" s="5" t="n">
         <v>0</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
@@ -2037,13 +2037,13 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>76.2</v>
+        <v>75.62</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="I18" s="4" t="n">
         <v>15.5</v>
@@ -2058,10 +2058,10 @@
         <v>0.55</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>29.6</v>
+        <v>29.8</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>0</v>
@@ -2085,86 +2085,90 @@
       <c r="T18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>ERF.PA</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Eurofins Scientific</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>NON CONFORME</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>69</v>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Ratio dette : 40.5% &gt; 33%</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>62.02</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="H19" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="I19" s="6" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="M19" s="6" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="O19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="6" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S19" s="6" t="inlineStr">
-        <is>
-          <t>Diagnostics &amp; Research</t>
-        </is>
-      </c>
-      <c r="T19" s="6" t="inlineStr"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>BN.PA</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Danone</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>CONFORME ⚠️</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Tous les critères AAOIFI respectés</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>71.92</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>Packaged Foods</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>Vérifier si produits à base de porc ou gélatine porcine</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>ALO.PA</t>
+          <t>ERF.PA</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Schneider Electric</t>
+          <t>Eurofins Scientific</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2173,39 +2177,39 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 35.3% &gt; 33%</t>
+          <t>Ratio dette : 40.8% &gt; 33%</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>23.84</v>
+        <v>61.48</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>41.1</v>
+        <v>24.1</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>3.3</v>
+        <v>9.5</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.7</v>
+        <v>6.5</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>1.27</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>35.3</v>
+        <v>40.8</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>15.3</v>
+        <v>7.3</v>
       </c>
       <c r="O20" s="6" t="n">
         <v>0</v>
@@ -2218,12 +2222,12 @@
       </c>
       <c r="R20" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="S20" s="6" t="inlineStr">
         <is>
-          <t>Railroads</t>
+          <t>Diagnostics &amp; Research</t>
         </is>
       </c>
       <c r="T20" s="6" t="inlineStr"/>
@@ -2231,12 +2235,12 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>MT.AS</t>
+          <t>ALO.PA</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>ArcelorMittal</t>
+          <t>Schneider Electric</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -2249,35 +2253,35 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 38.6% &gt; 33%</t>
+          <t>Ratio dette : 36.1% &gt; 33%</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>45.64</v>
+        <v>23.3</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>12.9</v>
+        <v>40.2</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>6</v>
+        <v>3.3</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>5.1</v>
+        <v>1.7</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1.7</v>
+        <v>3.2</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>1.67</v>
+        <v>1.27</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>38.6</v>
+        <v>36.1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>15.5</v>
+        <v>15.7</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>0</v>
@@ -2290,12 +2294,12 @@
       </c>
       <c r="R21" s="6" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="S21" s="6" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Railroads</t>
         </is>
       </c>
       <c r="T21" s="6" t="inlineStr"/>
@@ -2303,12 +2307,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>TTE.PA</t>
+          <t>MT.AS</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>ArcelorMittal</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -2317,39 +2321,39 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 41.4% &gt; 33%</t>
+          <t>Ratio dette : 39.4% &gt; 33%</t>
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>69.83</v>
+        <v>44.73</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>14</v>
+        <v>12.6</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>486</v>
+        <v>108</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>11.2</v>
+        <v>6</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>7.2</v>
+        <v>5.1</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>-2.5</v>
+        <v>1.7</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>0.28</v>
+        <v>1.67</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>41.4</v>
+        <v>39.4</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>19.9</v>
+        <v>15.8</v>
       </c>
       <c r="O22" s="6" t="n">
         <v>0</v>
@@ -2362,12 +2366,12 @@
       </c>
       <c r="R22" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="S22" s="6" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Integrated</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="T22" s="6" t="inlineStr"/>
@@ -2375,12 +2379,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>SGO.PA</t>
+          <t>TTE.PA</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Saint-Gobain</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -2389,39 +2393,39 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 50.2% &gt; 33%</t>
+          <t>Ratio dette : 40.0% &gt; 33%</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>72.62</v>
+        <v>72.33</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>12.9</v>
+        <v>14.4</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>311</v>
+        <v>483</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>11.7</v>
+        <v>11.2</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>6.2</v>
+        <v>7.2</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>-2.1</v>
+        <v>-2.5</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>1.14</v>
+        <v>0.28</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>50.2</v>
+        <v>40</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>21.5</v>
+        <v>19.2</v>
       </c>
       <c r="O23" s="6" t="n">
         <v>0</v>
@@ -2434,12 +2438,12 @@
       </c>
       <c r="R23" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="S23" s="6" t="inlineStr">
         <is>
-          <t>Building Products &amp; Equipment</t>
+          <t>Oil &amp; Gas Integrated</t>
         </is>
       </c>
       <c r="T23" s="6" t="inlineStr"/>
@@ -2447,12 +2451,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>DG.PA</t>
+          <t>SGO.PA</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Vinci</t>
+          <t>Saint-Gobain</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -2461,39 +2465,39 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 56.7% &gt; 33%</t>
+          <t>Ratio dette : 50.8% &gt; 33%</t>
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>129.55</v>
+        <v>71.8</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>15</v>
+        <v>12.8</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>383</v>
+        <v>318</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>15.4</v>
+        <v>11.7</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>5.2</v>
+        <v>-2.1</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>0.79</v>
+        <v>1.14</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>56.7</v>
+        <v>50.8</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>25.7</v>
+        <v>21.3</v>
       </c>
       <c r="O24" s="6" t="n">
         <v>0</v>
@@ -2511,7 +2515,7 @@
       </c>
       <c r="S24" s="6" t="inlineStr">
         <is>
-          <t>Engineering &amp; Construction</t>
+          <t>Building Products &amp; Equipment</t>
         </is>
       </c>
       <c r="T24" s="6" t="inlineStr"/>
@@ -2537,11 +2541,11 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 101.0% &gt; 33%</t>
+          <t>Ratio dette : 102.1% &gt; 33%</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -2549,7 +2553,7 @@
         </is>
       </c>
       <c r="H25" s="6" t="n">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>-1.4</v>
@@ -2564,10 +2568,10 @@
         <v>1.16</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>101</v>
+        <v>102.1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="O25" s="6" t="n">
         <v>0</v>
@@ -2597,53 +2601,53 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>BN.PA</t>
+          <t>DG.PA</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Danone</t>
+          <t>Vinci</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>NON CONFORME ⚠️</t>
+          <t>NON CONFORME</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 33.8% &gt; 33%</t>
+          <t>Ratio dette : 56.8% &gt; 33%</t>
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>69.86</v>
+        <v>129.35</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>24.8</v>
+        <v>15</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>326</v>
+        <v>385</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>10.8</v>
+        <v>15.4</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>-0.5</v>
+        <v>5.2</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>0.21</v>
+        <v>0.79</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>33.8</v>
+        <v>56.8</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>14.7</v>
+        <v>25.8</v>
       </c>
       <c r="O26" s="6" t="n">
         <v>0</v>
@@ -2656,19 +2660,15 @@
       </c>
       <c r="R26" s="6" t="inlineStr">
         <is>
-          <t>Consumer Defensive</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="S26" s="6" t="inlineStr">
         <is>
-          <t>Packaged Foods</t>
-        </is>
-      </c>
-      <c r="T26" s="6" t="inlineStr">
-        <is>
-          <t>Vérifier si produits à base de porc ou gélatine porcine</t>
-        </is>
-      </c>
+          <t>Engineering &amp; Construction</t>
+        </is>
+      </c>
+      <c r="T26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -2687,21 +2687,21 @@
         </is>
       </c>
       <c r="D27" s="6" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 83.0% &gt; 33%</t>
+          <t>Ratio dette : 78.7% &gt; 33%</t>
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>27.36</v>
+        <v>27.64</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="I27" s="6" t="n">
         <v>11.5</v>
@@ -2716,10 +2716,10 @@
         <v>0.62</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>83</v>
+        <v>78.7</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>29</v>
+        <v>27.5</v>
       </c>
       <c r="O27" s="6" t="n">
         <v>0</v>
@@ -2763,14 +2763,14 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 80.1% &gt; 33%</t>
+          <t>Ratio dette : 79.3% &gt; 33%</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>49.32</v>
+        <v>49.81</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>17.9</v>
+        <v>18.1</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>424</v>
@@ -2788,10 +2788,10 @@
         <v>0.72</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>80.09999999999999</v>
+        <v>79.3</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>39.8</v>
+        <v>39.4</v>
       </c>
       <c r="O28" s="6" t="n">
         <v>0</v>
@@ -2835,17 +2835,17 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 101.6% &gt; 33%</t>
+          <t>Ratio dette : 98.3% &gt; 33%</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
-        <v>16.95</v>
+        <v>17.52</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>84.8</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>3.2</v>
@@ -2860,10 +2860,10 @@
         <v>0.25</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>101.6</v>
+        <v>98.3</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>33.9</v>
+        <v>32.8</v>
       </c>
       <c r="O29" s="6" t="n">
         <v>0</v>
@@ -2907,11 +2907,11 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 841.5% &gt; 33%</t>
+          <t>Ratio dette : 852.5% &gt; 33%</t>
         </is>
       </c>
       <c r="F30" s="6" t="n">
-        <v>28.84</v>
+        <v>28.47</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="H30" s="6" t="n">
-        <v>761</v>
+        <v>755</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>-40.4</v>
@@ -2934,10 +2934,10 @@
         <v>0.78</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>841.5</v>
+        <v>852.5</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>243.5</v>
+        <v>246.7</v>
       </c>
       <c r="O30" s="6" t="n">
         <v>0</v>
@@ -2981,11 +2981,11 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 274.6% &gt; 33%</t>
+          <t>Ratio dette : 277.9% &gt; 33%</t>
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>5.78</v>
+        <v>5.71</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
@@ -3008,10 +3008,10 @@
         <v>0.98</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>274.6</v>
+        <v>277.9</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>175.4</v>
+        <v>177.5</v>
       </c>
       <c r="O31" s="6" t="n">
         <v>0</v>
@@ -3055,17 +3055,17 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 167.7% &gt; 33%</t>
+          <t>Ratio dette : 166.8% &gt; 33%</t>
         </is>
       </c>
       <c r="F32" s="6" t="n">
-        <v>50.98</v>
+        <v>51.24</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>6.1</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>867</v>
+        <v>885</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>11.5</v>
@@ -3080,10 +3080,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>167.7</v>
+        <v>166.8</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>33.6</v>
+        <v>33.4</v>
       </c>
       <c r="O32" s="6" t="n">
         <v>0</v>
@@ -3127,17 +3127,17 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 122.3% &gt; 33%</t>
+          <t>Ratio dette : 122.6% &gt; 33%</t>
         </is>
       </c>
       <c r="F33" s="6" t="n">
-        <v>32.99</v>
+        <v>32.92</v>
       </c>
       <c r="G33" s="6" t="n">
         <v>19.4</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>12.2</v>
@@ -3152,10 +3152,10 @@
         <v>1.04</v>
       </c>
       <c r="M33" s="6" t="n">
-        <v>122.3</v>
+        <v>122.6</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="O33" s="6" t="n">
         <v>0</v>
@@ -3199,11 +3199,11 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 699.6% &gt; 33%</t>
+          <t>Ratio dette : 676.5% &gt; 33%</t>
         </is>
       </c>
       <c r="F34" s="6" t="n">
-        <v>1.58</v>
+        <v>0.37</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
@@ -3226,10 +3226,10 @@
         <v>1.13</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>699.6</v>
+        <v>676.5</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>202.7</v>
+        <v>196</v>
       </c>
       <c r="O34" s="6" t="n">
         <v>0</v>
@@ -3273,17 +3273,17 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Ratio dette : 193.8% &gt; 33%</t>
+          <t>Ratio dette : 192.5% &gt; 33%</t>
         </is>
       </c>
       <c r="F35" s="6" t="n">
-        <v>15.39</v>
+        <v>15.5</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>639</v>
+        <v>629</v>
       </c>
       <c r="I35" s="6" t="n">
         <v>8.6</v>
@@ -3298,10 +3298,10 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M35" s="6" t="n">
-        <v>193.8</v>
+        <v>192.5</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>58.5</v>
+        <v>58.1</v>
       </c>
       <c r="O35" s="6" t="n">
         <v>0</v>
@@ -3353,13 +3353,13 @@
         </is>
       </c>
       <c r="F36" s="7" t="n">
-        <v>37.96</v>
+        <v>38.3</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>612</v>
+        <v>608</v>
       </c>
       <c r="I36" s="7" t="n">
         <v>18.1</v>
@@ -3433,13 +3433,13 @@
         </is>
       </c>
       <c r="F37" s="7" t="n">
-        <v>86.3</v>
+        <v>84.89</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>1112</v>
+        <v>1160</v>
       </c>
       <c r="I37" s="7" t="n">
         <v>9.699999999999999</v>
@@ -3513,13 +3513,13 @@
         </is>
       </c>
       <c r="F38" s="7" t="n">
-        <v>16.46</v>
+        <v>16.32</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>664</v>
+        <v>684</v>
       </c>
       <c r="I38" s="7" t="n">
         <v>6.9</v>
@@ -3593,7 +3593,7 @@
         </is>
       </c>
       <c r="F39" s="7" t="n">
-        <v>253.05</v>
+        <v>248.7</v>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="H39" s="7" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I39" s="7" t="n">
         <v>0.2</v>
@@ -3675,13 +3675,13 @@
         </is>
       </c>
       <c r="F40" s="7" t="n">
-        <v>494.1</v>
+        <v>473.7</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>22.6</v>
+        <v>21.7</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="I40" s="7" t="n">
         <v>16.2</v>
@@ -3755,13 +3755,13 @@
         </is>
       </c>
       <c r="F41" s="7" t="n">
-        <v>69.59999999999999</v>
+        <v>68.52</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>656</v>
+        <v>686</v>
       </c>
       <c r="I41" s="7" t="n">
         <v>8.6</v>
@@ -3835,13 +3835,13 @@
         </is>
       </c>
       <c r="F42" s="7" t="n">
-        <v>65</v>
+        <v>64.12</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>9.6</v>
+        <v>9.4</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>8.800000000000001</v>
@@ -3905,7 +3905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3994,20 +3994,22 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Unibail-Rodamco</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
         <v>100</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>109.5</v>
-      </c>
-      <c r="E3" s="12" t="n">
-        <v>12</v>
+        <v>0</v>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F3" s="12" t="n">
-        <v>316</v>
+        <v>0</v>
       </c>
       <c r="G3" s="12" t="n">
         <v>0</v>
@@ -4026,20 +4028,20 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Michelin</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
         <v>100</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>29.78</v>
+        <v>107.8</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>2.9</v>
+        <v>11.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0</v>
+        <v>316</v>
       </c>
       <c r="G4" s="12" t="n">
         <v>0</v>
@@ -4058,19 +4060,17 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Unibail-Rodamco</t>
+          <t>Michelin</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
         <v>100</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>29.66</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>2.9</v>
       </c>
       <c r="F5" s="12" t="n">
         <v>0</v>
@@ -4099,13 +4099,13 @@
         <v>94</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>1908</v>
+        <v>1873</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>44.4</v>
+        <v>43.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G6" s="12" t="n">
         <v>25.2</v>
@@ -4131,19 +4131,19 @@
         <v>91</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>361.25</v>
+        <v>353.65</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>31.6</v>
+        <v>31</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G7" s="12" t="n">
         <v>18</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="I7" s="12" t="n">
         <v>0</v>
@@ -4163,19 +4163,19 @@
         <v>87</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>252.2</v>
+        <v>248</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>31.7</v>
+        <v>31.1</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G8" s="12" t="n">
         <v>15.6</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>14</v>
+        <v>14.3</v>
       </c>
       <c r="I8" s="12" t="n">
         <v>0</v>
@@ -4192,22 +4192,22 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>169.16</v>
+        <v>170.88</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>27.7</v>
+        <v>28</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="G9" s="12" t="n">
         <v>13.4</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>14</v>
+        <v>13.8</v>
       </c>
       <c r="I9" s="12" t="n">
         <v>0</v>
@@ -4227,10 +4227,10 @@
         <v>86</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>209.5</v>
+        <v>204.7</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>42.1</v>
+        <v>41.2</v>
       </c>
       <c r="F10" s="12" t="n">
         <v>190</v>
@@ -4239,7 +4239,7 @@
         <v>6.1</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>14.8</v>
+        <v>15.2</v>
       </c>
       <c r="I10" s="12" t="n">
         <v>0</v>
@@ -4259,13 +4259,13 @@
         <v>83</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>306.1</v>
+        <v>304.4</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>55.6</v>
@@ -4295,10 +4295,10 @@
         <v>81</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>137.6</v>
+        <v>136.85</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>29.3</v>
+        <v>29.1</v>
       </c>
       <c r="F12" s="12" t="n">
         <v>172</v>
@@ -4307,7 +4307,7 @@
         <v>16.8</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="I12" s="12" t="n">
         <v>0</v>
@@ -4327,19 +4327,19 @@
         <v>79</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>18.61</v>
+        <v>18.5</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G13" s="12" t="n">
         <v>13.3</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
       <c r="I13" s="12" t="n">
         <v>0</v>
@@ -4359,19 +4359,19 @@
         <v>78</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>28.91</v>
+        <v>28.61</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>192.7</v>
+        <v>178.8</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G14" s="12" t="n">
         <v>1</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I14" s="12" t="n">
         <v>0</v>
@@ -4391,13 +4391,13 @@
         <v>77</v>
       </c>
       <c r="D15" s="12" t="n">
-        <v>76.41</v>
+        <v>76.39</v>
       </c>
       <c r="E15" s="12" t="n">
         <v>19</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="G15" s="12" t="n">
         <v>6.7</v>
@@ -4423,19 +4423,19 @@
         <v>75</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>255.1</v>
+        <v>253.8</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>31.4</v>
+        <v>31.2</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>21.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="I16" s="14" t="n">
         <v>0</v>
@@ -4459,19 +4459,19 @@
         <v>72</v>
       </c>
       <c r="D17" s="14" t="n">
-        <v>171.3</v>
+        <v>168.38</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>21.6</v>
       </c>
       <c r="H17" s="14" t="n">
-        <v>10.5</v>
+        <v>10.7</v>
       </c>
       <c r="I17" s="14" t="n">
         <v>0</v>
@@ -4492,27 +4492,63 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>76.2</v>
+        <v>75.62</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G18" s="12" t="n">
         <v>15.5</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>29.6</v>
+        <v>29.8</v>
       </c>
       <c r="I18" s="12" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Danone</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>54</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>71.92</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>Vérifier si produits à base de porc ou gélatine porcine</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4529,7 +4565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4551,7 +4587,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -4561,7 +4597,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -4589,7 +4625,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Unibail-Rodamco</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4599,7 +4635,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Michelin</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4609,7 +4645,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Unibail-Rodamco</t>
+          <t>Michelin</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4653,7 +4689,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15">
@@ -4743,7 +4779,17 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>62</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Danone</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>